<commit_message>
New Test Cases, New approach, running from Ecxel sheet,etc.
</commit_message>
<xml_diff>
--- a/TestData/Convert_TestData.xlsx
+++ b/TestData/Convert_TestData.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -490,6 +490,376 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>HKD into every wallet</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>lawma195.infinity@gmail.com</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>12345678</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Convert successfully!</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PHP into every wallet</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>lawma195.infinity@gmail.com</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>12345678</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>PHP</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Convert successfully!</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BDT into every wallet</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>lawma195.infinity@gmail.com</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>12345678</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>BDT</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Convert successfully!</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>VND into every wallet</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>lawma195.infinity@gmail.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>12345678</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Convert successfully!</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>IDR into every wallet</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>lawma195.infinity@gmail.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>12345678</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>IDR</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Convert successfully!</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MYR into every wallet</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>lawma195.infinity@gmail.com</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>12345678</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>MYR</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Convert successfully!</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>USD into every wallet</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>lawma195.infinity@gmail.com</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>12345678</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Convert successfully!</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BRL into every wallet</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>lawma195.infinity@gmail.com</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>12345678</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>BRL</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Convert successfully!</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MXN into every wallet</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>lawma195.infinity@gmail.com</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>12345678</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Convert successfully!</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>THB into every wallet</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>lawma195.infinity@gmail.com</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>12345678</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Convert successfully!</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>